<commit_message>
implement gt and llm reports
</commit_message>
<xml_diff>
--- a/outputs/evaluation/CF_M01_req_eval_gt_report.xlsx
+++ b/outputs/evaluation/CF_M01_req_eval_gt_report.xlsx
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>0.3483</v>
+        <v>0.3481</v>
       </c>
     </row>
     <row r="3">
@@ -548,7 +548,7 @@
         </is>
       </c>
       <c r="K3" t="n">
-        <v>0.2428</v>
+        <v>0.2434</v>
       </c>
     </row>
     <row r="4">
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>0.3222</v>
+        <v>0.3186</v>
       </c>
     </row>
     <row r="5">
@@ -618,11 +618,11 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>The system shall allow users with permissions to list the different connections of the players in the system.</t>
+          <t>The system shall allow users with permissions to list the different player connections of the system.</t>
         </is>
       </c>
       <c r="K5" t="n">
-        <v>0.2979</v>
+        <v>0.2574</v>
       </c>
     </row>
     <row r="6">
@@ -659,7 +659,7 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>0.2963</v>
+        <v>0.2969</v>
       </c>
     </row>
   </sheetData>

</xml_diff>